<commit_message>
Phase 2: add FF core script, overlay script, rest features, experimental scripts. Phase 1: add 2026-03-24 workbook.
</commit_message>
<xml_diff>
--- a/NCAAB Excel & Python Predictive & Pricing Model/Phase 1/ncaab_market_maker_2026-03-24_PRODUCTION.xlsx
+++ b/NCAAB Excel & Python Predictive & Pricing Model/Phase 1/ncaab_market_maker_2026-03-24_PRODUCTION.xlsx
@@ -2091,40 +2091,40 @@
         <v>174.5</v>
       </c>
       <c r="H3" s="52" t="n">
-        <v>3.732</v>
+        <v>3.939</v>
       </c>
       <c r="I3" s="51" t="n">
-        <v>165.462</v>
+        <v>166.095</v>
       </c>
       <c r="J3" s="52" t="n">
-        <v>3.732</v>
+        <v>3.939</v>
       </c>
       <c r="K3" s="44" t="n">
-        <v>0.5862000000000001</v>
+        <v>0.5915</v>
       </c>
       <c r="L3" s="40" t="n">
-        <v>0.3229</v>
+        <v>0.3283</v>
       </c>
       <c r="M3" s="47" t="n">
-        <v>0.318</v>
+        <v>0.3292</v>
       </c>
       <c r="N3" s="53" t="n">
-        <v>-142</v>
+        <v>-145</v>
       </c>
       <c r="O3" s="44" t="n">
-        <v>0.5862000000000001</v>
+        <v>0.5915</v>
       </c>
       <c r="P3" s="40" t="n">
-        <v>0.3229</v>
+        <v>0.3283</v>
       </c>
       <c r="Q3" s="47" t="n">
-        <v>0.318</v>
+        <v>0.3292</v>
       </c>
       <c r="R3" s="53" t="n">
-        <v>-142</v>
+        <v>-145</v>
       </c>
       <c r="S3" s="54" t="n">
-        <v>-6.268</v>
+        <v>-6.061</v>
       </c>
       <c r="T3" s="24" t="inlineStr">
         <is>
@@ -2175,40 +2175,40 @@
         <v>168</v>
       </c>
       <c r="H4" s="57" t="n">
-        <v>-4.806</v>
+        <v>-5.134</v>
       </c>
       <c r="I4" s="56" t="n">
-        <v>161.874</v>
+        <v>162.616</v>
       </c>
       <c r="J4" s="57" t="n">
-        <v>-4.806</v>
+        <v>-5.134</v>
       </c>
       <c r="K4" s="58" t="n">
-        <v>0.3584</v>
+        <v>0.3504</v>
       </c>
       <c r="L4" s="36" t="n">
-        <v>0.5741000000000001</v>
+        <v>0.5651</v>
       </c>
       <c r="M4" s="58" t="n">
-        <v>0.3576</v>
+        <v>0.3716</v>
       </c>
       <c r="N4" s="59" t="n">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="O4" s="58" t="n">
-        <v>0.3584</v>
+        <v>0.3504</v>
       </c>
       <c r="P4" s="36" t="n">
-        <v>0.5741000000000001</v>
+        <v>0.5651</v>
       </c>
       <c r="Q4" s="58" t="n">
-        <v>0.3576</v>
+        <v>0.3716</v>
       </c>
       <c r="R4" s="59" t="n">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="S4" s="60" t="n">
-        <v>3.194</v>
+        <v>2.866</v>
       </c>
       <c r="T4" s="18" t="inlineStr">
         <is>
@@ -2259,40 +2259,40 @@
         <v>154.5</v>
       </c>
       <c r="H5" s="61" t="n">
-        <v>-2.241</v>
+        <v>-2.259</v>
       </c>
       <c r="I5" s="51" t="n">
-        <v>152.67</v>
+        <v>153.457</v>
       </c>
       <c r="J5" s="61" t="n">
-        <v>-2.241</v>
+        <v>-2.259</v>
       </c>
       <c r="K5" s="47" t="n">
-        <v>0.423</v>
+        <v>0.4228</v>
       </c>
       <c r="L5" s="40" t="n">
-        <v>0.6976</v>
+        <v>0.6966</v>
       </c>
       <c r="M5" s="40" t="n">
-        <v>0.4463</v>
+        <v>0.4626</v>
       </c>
       <c r="N5" s="53" t="n">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="O5" s="47" t="n">
-        <v>0.423</v>
+        <v>0.4228</v>
       </c>
       <c r="P5" s="40" t="n">
-        <v>0.6976</v>
+        <v>0.6966</v>
       </c>
       <c r="Q5" s="40" t="n">
-        <v>0.4463</v>
+        <v>0.4626</v>
       </c>
       <c r="R5" s="53" t="n">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="S5" s="54" t="n">
-        <v>7.259</v>
+        <v>7.241</v>
       </c>
       <c r="T5" s="24" t="inlineStr">
         <is>
@@ -2343,40 +2343,40 @@
         <v>147</v>
       </c>
       <c r="H6" s="57" t="n">
-        <v>-2.381</v>
+        <v>-2.465</v>
       </c>
       <c r="I6" s="56" t="n">
-        <v>147.667</v>
+        <v>148.332</v>
       </c>
       <c r="J6" s="57" t="n">
-        <v>-2.381</v>
+        <v>-2.465</v>
       </c>
       <c r="K6" s="58" t="n">
-        <v>0.4175</v>
+        <v>0.4154</v>
       </c>
       <c r="L6" s="36" t="n">
-        <v>0.5329</v>
+        <v>0.5304</v>
       </c>
       <c r="M6" s="36" t="n">
-        <v>0.4877</v>
+        <v>0.5018</v>
       </c>
       <c r="N6" s="59" t="n">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="O6" s="58" t="n">
-        <v>0.4175</v>
+        <v>0.4154</v>
       </c>
       <c r="P6" s="36" t="n">
-        <v>0.5329</v>
+        <v>0.5304</v>
       </c>
       <c r="Q6" s="36" t="n">
-        <v>0.4877</v>
+        <v>0.5018</v>
       </c>
       <c r="R6" s="59" t="n">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="S6" s="60" t="n">
-        <v>1.119</v>
+        <v>1.035</v>
       </c>
       <c r="T6" s="18" t="inlineStr">
         <is>
@@ -2427,40 +2427,40 @@
         <v>162</v>
       </c>
       <c r="H7" s="52" t="n">
-        <v>3.767</v>
+        <v>4.322</v>
       </c>
       <c r="I7" s="51" t="n">
-        <v>156.953</v>
+        <v>157.892</v>
       </c>
       <c r="J7" s="52" t="n">
-        <v>3.767</v>
+        <v>4.322</v>
       </c>
       <c r="K7" s="44" t="n">
-        <v>0.5898</v>
+        <v>0.6044</v>
       </c>
       <c r="L7" s="40" t="n">
-        <v>0.4235</v>
+        <v>0.4389</v>
       </c>
       <c r="M7" s="47" t="n">
-        <v>0.3747</v>
+        <v>0.393</v>
       </c>
       <c r="N7" s="53" t="n">
-        <v>-144</v>
+        <v>-153</v>
       </c>
       <c r="O7" s="44" t="n">
-        <v>0.5898</v>
+        <v>0.6044</v>
       </c>
       <c r="P7" s="40" t="n">
-        <v>0.4235</v>
+        <v>0.4389</v>
       </c>
       <c r="Q7" s="47" t="n">
-        <v>0.3747</v>
+        <v>0.393</v>
       </c>
       <c r="R7" s="53" t="n">
-        <v>-144</v>
+        <v>-153</v>
       </c>
       <c r="S7" s="54" t="n">
-        <v>-2.233</v>
+        <v>-1.678</v>
       </c>
       <c r="T7" s="24" t="inlineStr">
         <is>
@@ -2511,40 +2511,40 @@
         <v>148.5</v>
       </c>
       <c r="H8" s="57" t="n">
-        <v>-2.623</v>
+        <v>-2.498</v>
       </c>
       <c r="I8" s="56" t="n">
-        <v>147.219</v>
+        <v>147.377</v>
       </c>
       <c r="J8" s="57" t="n">
-        <v>-2.623</v>
+        <v>-2.498</v>
       </c>
       <c r="K8" s="58" t="n">
-        <v>0.4105</v>
+        <v>0.4141</v>
       </c>
       <c r="L8" s="36" t="n">
-        <v>0.497</v>
+        <v>0.5006</v>
       </c>
       <c r="M8" s="36" t="n">
-        <v>0.4568</v>
+        <v>0.4602</v>
       </c>
       <c r="N8" s="59" t="n">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="O8" s="58" t="n">
-        <v>0.4105</v>
+        <v>0.4141</v>
       </c>
       <c r="P8" s="36" t="n">
-        <v>0.497</v>
+        <v>0.5006</v>
       </c>
       <c r="Q8" s="36" t="n">
-        <v>0.4568</v>
+        <v>0.4602</v>
       </c>
       <c r="R8" s="59" t="n">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="S8" s="60" t="n">
-        <v>-0.123</v>
+        <v>0.002</v>
       </c>
       <c r="T8" s="18" t="inlineStr">
         <is>
@@ -2595,40 +2595,40 @@
         <v>139</v>
       </c>
       <c r="H9" s="61" t="n">
-        <v>-1.977</v>
+        <v>-2.21</v>
       </c>
       <c r="I9" s="51" t="n">
-        <v>141.116</v>
+        <v>141.2</v>
       </c>
       <c r="J9" s="61" t="n">
-        <v>-1.977</v>
+        <v>-2.21</v>
       </c>
       <c r="K9" s="47" t="n">
-        <v>0.427</v>
+        <v>0.4202</v>
       </c>
       <c r="L9" s="40" t="n">
-        <v>0.6604</v>
+        <v>0.654</v>
       </c>
       <c r="M9" s="40" t="n">
-        <v>0.52</v>
+        <v>0.5219</v>
       </c>
       <c r="N9" s="53" t="n">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="O9" s="47" t="n">
-        <v>0.427</v>
+        <v>0.4202</v>
       </c>
       <c r="P9" s="40" t="n">
-        <v>0.6604</v>
+        <v>0.654</v>
       </c>
       <c r="Q9" s="40" t="n">
-        <v>0.52</v>
+        <v>0.5219</v>
       </c>
       <c r="R9" s="53" t="n">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="S9" s="54" t="n">
-        <v>5.523</v>
+        <v>5.29</v>
       </c>
       <c r="T9" s="24" t="inlineStr">
         <is>
@@ -2679,40 +2679,40 @@
         <v>142</v>
       </c>
       <c r="H10" s="57" t="n">
-        <v>-4.579</v>
+        <v>-4.734</v>
       </c>
       <c r="I10" s="56" t="n">
-        <v>146.136</v>
+        <v>146.096</v>
       </c>
       <c r="J10" s="57" t="n">
-        <v>-4.579</v>
+        <v>-4.734</v>
       </c>
       <c r="K10" s="58" t="n">
-        <v>0.3559</v>
+        <v>0.3517</v>
       </c>
       <c r="L10" s="36" t="n">
-        <v>0.5568</v>
+        <v>0.5524</v>
       </c>
       <c r="M10" s="36" t="n">
-        <v>0.5628</v>
+        <v>0.5619</v>
       </c>
       <c r="N10" s="59" t="n">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="O10" s="58" t="n">
-        <v>0.3559</v>
+        <v>0.3517</v>
       </c>
       <c r="P10" s="36" t="n">
-        <v>0.5568</v>
+        <v>0.5524</v>
       </c>
       <c r="Q10" s="36" t="n">
-        <v>0.5628</v>
+        <v>0.5619</v>
       </c>
       <c r="R10" s="59" t="n">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="S10" s="60" t="n">
-        <v>1.921</v>
+        <v>1.766</v>
       </c>
       <c r="T10" s="18" t="inlineStr">
         <is>
@@ -2762,41 +2762,41 @@
       <c r="G11" s="51" t="n">
         <v>140</v>
       </c>
-      <c r="H11" s="52" t="n">
-        <v>0.207</v>
+      <c r="H11" s="61" t="n">
+        <v>-0.01</v>
       </c>
       <c r="I11" s="51" t="n">
-        <v>146.95</v>
-      </c>
-      <c r="J11" s="52" t="n">
-        <v>0.207</v>
+        <v>147.307</v>
+      </c>
+      <c r="J11" s="61" t="n">
+        <v>-0.01</v>
       </c>
       <c r="K11" s="40" t="n">
-        <v>0.4914</v>
+        <v>0.4852</v>
       </c>
       <c r="L11" s="40" t="n">
-        <v>0.6065</v>
+        <v>0.6002999999999999</v>
       </c>
       <c r="M11" s="44" t="n">
-        <v>0.6224</v>
+        <v>0.6296</v>
       </c>
       <c r="N11" s="53" t="n">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="O11" s="40" t="n">
-        <v>0.4914</v>
+        <v>0.4852</v>
       </c>
       <c r="P11" s="40" t="n">
-        <v>0.6065</v>
+        <v>0.6002999999999999</v>
       </c>
       <c r="Q11" s="44" t="n">
-        <v>0.6224</v>
+        <v>0.6296</v>
       </c>
       <c r="R11" s="53" t="n">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="S11" s="54" t="n">
-        <v>3.707</v>
+        <v>3.49</v>
       </c>
       <c r="T11" s="24" t="inlineStr">
         <is>
@@ -2847,40 +2847,40 @@
         <v>134</v>
       </c>
       <c r="H12" s="62" t="n">
-        <v>1.201</v>
+        <v>1.334</v>
       </c>
       <c r="I12" s="56" t="n">
-        <v>140.532</v>
+        <v>140.666</v>
       </c>
       <c r="J12" s="62" t="n">
-        <v>1.201</v>
+        <v>1.334</v>
       </c>
       <c r="K12" s="36" t="n">
-        <v>0.5207000000000001</v>
+        <v>0.5246</v>
       </c>
       <c r="L12" s="36" t="n">
-        <v>0.4908</v>
+        <v>0.4948</v>
       </c>
       <c r="M12" s="46" t="n">
-        <v>0.6181</v>
+        <v>0.621</v>
       </c>
       <c r="N12" s="59" t="n">
-        <v>-109</v>
+        <v>-110</v>
       </c>
       <c r="O12" s="36" t="n">
-        <v>0.5207000000000001</v>
+        <v>0.5246</v>
       </c>
       <c r="P12" s="36" t="n">
-        <v>0.4908</v>
+        <v>0.4948</v>
       </c>
       <c r="Q12" s="46" t="n">
-        <v>0.6181</v>
+        <v>0.621</v>
       </c>
       <c r="R12" s="59" t="n">
-        <v>-109</v>
+        <v>-110</v>
       </c>
       <c r="S12" s="60" t="n">
-        <v>-0.299</v>
+        <v>-0.166</v>
       </c>
       <c r="T12" s="18" t="inlineStr">
         <is>
@@ -2931,40 +2931,40 @@
         <v>138.5</v>
       </c>
       <c r="H13" s="61" t="n">
-        <v>-2.916</v>
+        <v>-3.332</v>
       </c>
       <c r="I13" s="51" t="n">
-        <v>144.298</v>
+        <v>144.549</v>
       </c>
       <c r="J13" s="61" t="n">
-        <v>-2.916</v>
+        <v>-3.332</v>
       </c>
       <c r="K13" s="47" t="n">
-        <v>0.4011</v>
+        <v>0.3895</v>
       </c>
       <c r="L13" s="40" t="n">
-        <v>0.5471</v>
+        <v>0.535</v>
       </c>
       <c r="M13" s="44" t="n">
-        <v>0.6104000000000001</v>
+        <v>0.6156</v>
       </c>
       <c r="N13" s="53" t="n">
-        <v>149</v>
+        <v>157</v>
       </c>
       <c r="O13" s="47" t="n">
-        <v>0.4011</v>
+        <v>0.3895</v>
       </c>
       <c r="P13" s="40" t="n">
-        <v>0.5471</v>
+        <v>0.535</v>
       </c>
       <c r="Q13" s="44" t="n">
-        <v>0.6104000000000001</v>
+        <v>0.6156</v>
       </c>
       <c r="R13" s="53" t="n">
-        <v>149</v>
+        <v>157</v>
       </c>
       <c r="S13" s="54" t="n">
-        <v>1.584</v>
+        <v>1.168</v>
       </c>
       <c r="T13" s="24" t="inlineStr">
         <is>
@@ -3014,41 +3014,41 @@
       <c r="G14" s="56" t="n">
         <v>136.5</v>
       </c>
-      <c r="H14" s="57" t="n">
-        <v>-0.117</v>
+      <c r="H14" s="62" t="n">
+        <v>0.107</v>
       </c>
       <c r="I14" s="56" t="n">
-        <v>144.254</v>
-      </c>
-      <c r="J14" s="57" t="n">
-        <v>-0.117</v>
+        <v>144.571</v>
+      </c>
+      <c r="J14" s="62" t="n">
+        <v>0.107</v>
       </c>
       <c r="K14" s="36" t="n">
-        <v>0.4819</v>
+        <v>0.4884</v>
       </c>
       <c r="L14" s="36" t="n">
-        <v>0.4235</v>
+        <v>0.43</v>
       </c>
       <c r="M14" s="46" t="n">
-        <v>0.6519</v>
+        <v>0.6582</v>
       </c>
       <c r="N14" s="59" t="n">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="O14" s="36" t="n">
-        <v>0.4819</v>
+        <v>0.4884</v>
       </c>
       <c r="P14" s="36" t="n">
-        <v>0.4235</v>
+        <v>0.43</v>
       </c>
       <c r="Q14" s="46" t="n">
-        <v>0.6519</v>
+        <v>0.6582</v>
       </c>
       <c r="R14" s="59" t="n">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="S14" s="60" t="n">
-        <v>-2.117</v>
+        <v>-1.893</v>
       </c>
       <c r="T14" s="18" t="inlineStr">
         <is>
@@ -3099,40 +3099,40 @@
         <v>152.75</v>
       </c>
       <c r="H15" s="61" t="n">
-        <v>-4.835</v>
+        <v>-5.193</v>
       </c>
       <c r="I15" s="51" t="n">
-        <v>147.55</v>
+        <v>147.555</v>
       </c>
       <c r="J15" s="61" t="n">
-        <v>-4.835</v>
+        <v>-5.193</v>
       </c>
       <c r="K15" s="47" t="n">
-        <v>0.3499</v>
+        <v>0.3403</v>
       </c>
       <c r="L15" s="40" t="n">
-        <v>0.6605</v>
+        <v>0.651</v>
       </c>
       <c r="M15" s="47" t="n">
-        <v>0.3812</v>
+        <v>0.3813</v>
       </c>
       <c r="N15" s="53" t="n">
-        <v>186</v>
+        <v>194</v>
       </c>
       <c r="O15" s="47" t="n">
-        <v>0.3499</v>
+        <v>0.3403</v>
       </c>
       <c r="P15" s="40" t="n">
-        <v>0.6605</v>
+        <v>0.651</v>
       </c>
       <c r="Q15" s="47" t="n">
-        <v>0.3812</v>
+        <v>0.3813</v>
       </c>
       <c r="R15" s="53" t="n">
-        <v>186</v>
+        <v>194</v>
       </c>
       <c r="S15" s="54" t="n">
-        <v>6.165</v>
+        <v>5.807</v>
       </c>
       <c r="T15" s="24" t="inlineStr">
         <is>
@@ -3183,40 +3183,40 @@
         <v>148.5</v>
       </c>
       <c r="H16" s="57" t="n">
-        <v>-5.585</v>
+        <v>-6.003</v>
       </c>
       <c r="I16" s="56" t="n">
-        <v>155.133</v>
+        <v>156.338</v>
       </c>
       <c r="J16" s="57" t="n">
-        <v>-5.585</v>
+        <v>-6.003</v>
       </c>
       <c r="K16" s="58" t="n">
-        <v>0.3348</v>
+        <v>0.3249</v>
       </c>
       <c r="L16" s="36" t="n">
-        <v>0.5268</v>
+        <v>0.515</v>
       </c>
       <c r="M16" s="46" t="n">
-        <v>0.6205000000000001</v>
+        <v>0.6437</v>
       </c>
       <c r="N16" s="59" t="n">
-        <v>199</v>
+        <v>208</v>
       </c>
       <c r="O16" s="58" t="n">
-        <v>0.3348</v>
+        <v>0.3249</v>
       </c>
       <c r="P16" s="36" t="n">
-        <v>0.5268</v>
+        <v>0.515</v>
       </c>
       <c r="Q16" s="46" t="n">
-        <v>0.6205000000000001</v>
+        <v>0.6437</v>
       </c>
       <c r="R16" s="59" t="n">
-        <v>199</v>
+        <v>208</v>
       </c>
       <c r="S16" s="60" t="n">
-        <v>1.415</v>
+        <v>0.997</v>
       </c>
       <c r="T16" s="18" t="inlineStr">
         <is>
@@ -3265,33 +3265,33 @@
         <v>134</v>
       </c>
       <c r="H17" s="61" t="n">
-        <v>-0.8139999999999999</v>
+        <v>-0.915</v>
       </c>
       <c r="I17" s="51" t="n">
-        <v>138.069</v>
+        <v>138.175</v>
       </c>
       <c r="J17" s="61" t="n">
-        <v>-0.8139999999999999</v>
+        <v>-0.915</v>
       </c>
       <c r="K17" s="40" t="n">
-        <v>0.4605</v>
+        <v>0.4575</v>
       </c>
       <c r="L17" s="40" t="inlineStr"/>
       <c r="M17" s="40" t="n">
-        <v>0.5649</v>
+        <v>0.5672</v>
       </c>
       <c r="N17" s="53" t="n">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="O17" s="40" t="n">
-        <v>0.4605</v>
+        <v>0.4575</v>
       </c>
       <c r="P17" s="40" t="inlineStr"/>
       <c r="Q17" s="40" t="n">
-        <v>0.5649</v>
+        <v>0.5672</v>
       </c>
       <c r="R17" s="53" t="n">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="S17" s="54" t="inlineStr"/>
       <c r="T17" s="24" t="inlineStr">
@@ -3343,40 +3343,40 @@
         <v>152.5</v>
       </c>
       <c r="H18" s="57" t="n">
-        <v>-1.564</v>
+        <v>-1.674</v>
       </c>
       <c r="I18" s="56" t="n">
-        <v>150.358</v>
+        <v>150.66</v>
       </c>
       <c r="J18" s="57" t="n">
-        <v>-1.564</v>
+        <v>-1.674</v>
       </c>
       <c r="K18" s="36" t="n">
-        <v>0.4413</v>
+        <v>0.4383</v>
       </c>
       <c r="L18" s="36" t="n">
-        <v>0.5839</v>
+        <v>0.5807</v>
       </c>
       <c r="M18" s="36" t="n">
-        <v>0.4394</v>
+        <v>0.4457</v>
       </c>
       <c r="N18" s="59" t="n">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="O18" s="36" t="n">
-        <v>0.4413</v>
+        <v>0.4383</v>
       </c>
       <c r="P18" s="36" t="n">
-        <v>0.5839</v>
+        <v>0.5807</v>
       </c>
       <c r="Q18" s="36" t="n">
-        <v>0.4394</v>
+        <v>0.4457</v>
       </c>
       <c r="R18" s="59" t="n">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="S18" s="60" t="n">
-        <v>2.686</v>
+        <v>2.576</v>
       </c>
       <c r="T18" s="18" t="inlineStr">
         <is>
@@ -3459,7 +3459,7 @@
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>2.836</t>
+          <t>3.057</t>
         </is>
       </c>
     </row>
@@ -3471,7 +3471,7 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>0.8868</t>
+          <t>0.8919</t>
         </is>
       </c>
     </row>
@@ -3483,7 +3483,7 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>3.041 pts</t>
+          <t>2.802 pts</t>
         </is>
       </c>
     </row>

</xml_diff>